<commit_message>
Updates to rubrics and lab instructions for winter 2026
</commit_message>
<xml_diff>
--- a/Labs/Lab06/Lab6Rubric_CS295N.xlsx
+++ b/Labs/Lab06/Lab6Rubric_CS295N.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/DataCard/Repos/CS295N-Repos/CS295N-CourseMaterials/Labs/Lab06/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Repos\CS295N-296N-Repos\CS295N-CourseMaterials\Labs\Lab06\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05AEA874-709F-D240-8C21-943103E2FC54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5B4A3EE-7C1D-4E30-B3F9-F2D4AC2B03F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10620" yWindow="540" windowWidth="15620" windowHeight="15460" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-15060" yWindow="4200" windowWidth="15048" windowHeight="12336" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Lab3Rubric_CS295N" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="35">
   <si>
     <t>-----------------------------------</t>
   </si>
@@ -120,9 +120,6 @@
     <t>A page showing all comments</t>
   </si>
   <si>
-    <t>Good start.</t>
-  </si>
-  <si>
     <t>Used correct style</t>
   </si>
   <si>
@@ -130,6 +127,18 @@
   </si>
   <si>
     <t>Option A</t>
+  </si>
+  <si>
+    <t>Part A, MVC Movie Tutorial</t>
+  </si>
+  <si>
+    <t>Exercise: Report (A, B, C) with screen-shot</t>
+  </si>
+  <si>
+    <t>Not required</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Excellent work! Good job of adding a database! </t>
   </si>
 </sst>
 </file>
@@ -675,7 +684,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
@@ -698,10 +707,28 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1058,12 +1085,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F61"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="16"/>
+  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6"/>
   <cols>
-    <col min="1" max="1" width="44.33203125" customWidth="1"/>
+    <col min="1" max="1" width="44.296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="19">
+    <row r="1" spans="1:6" ht="18">
       <c r="A1" s="5" t="s">
         <v>16</v>
       </c>
@@ -1086,7 +1113,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="18">
+    <row r="5" spans="1:6" ht="17.399999999999999">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -1183,7 +1210,7 @@
     </row>
     <row r="18" spans="1:6">
       <c r="A18" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B18">
         <v>2</v>
@@ -1327,7 +1354,7 @@
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B38">
         <v>2</v>
@@ -1490,7 +1517,7 @@
     </row>
     <row r="58" spans="1:3">
       <c r="A58" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B58">
         <v>2</v>
@@ -1536,12 +1563,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B8C8BAC4-7C35-B64C-9C0F-AC9B3324E891}">
   <dimension ref="A1:F69"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="16"/>
+  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6"/>
   <cols>
-    <col min="1" max="1" width="44.33203125" customWidth="1"/>
+    <col min="1" max="1" width="44.296875" customWidth="1"/>
+    <col min="2" max="2" width="7.19921875" customWidth="1"/>
+    <col min="3" max="3" width="5.8984375" customWidth="1"/>
+    <col min="4" max="4" width="17.09765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="19">
+    <row r="1" spans="1:6" ht="18">
       <c r="A1" s="5" t="s">
         <v>16</v>
       </c>
@@ -1557,16 +1587,19 @@
       </c>
     </row>
     <row r="4" spans="1:6">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="15" t="s">
         <v>12</v>
       </c>
+      <c r="B4" s="16"/>
+      <c r="C4" s="16"/>
+      <c r="D4" s="16"/>
     </row>
     <row r="5" spans="1:6">
       <c r="F5" s="6"/>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="4" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="B6" t="s">
         <v>2</v>
@@ -1578,28 +1611,32 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="18">
+    <row r="7" spans="1:6" ht="17.399999999999999">
       <c r="A7" t="s">
-        <v>5</v>
-      </c>
-      <c r="B7">
-        <v>10</v>
-      </c>
-      <c r="C7">
+        <v>32</v>
+      </c>
+      <c r="B7" s="17">
+        <v>10</v>
+      </c>
+      <c r="C7" s="17">
         <v>10</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F7" s="11"/>
     </row>
     <row r="8" spans="1:6">
+      <c r="B8" s="17"/>
+      <c r="C8" s="17"/>
       <c r="D8" s="13"/>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="4" t="s">
         <v>20</v>
       </c>
+      <c r="B9" s="17"/>
+      <c r="C9" s="17"/>
       <c r="D9" s="13"/>
       <c r="F9" s="6"/>
     </row>
@@ -1607,20 +1644,22 @@
       <c r="A10" t="s">
         <v>8</v>
       </c>
+      <c r="B10" s="17"/>
+      <c r="C10" s="17"/>
       <c r="D10" s="13"/>
     </row>
-    <row r="11" spans="1:6" ht="17">
+    <row r="11" spans="1:6">
       <c r="A11" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="12">
-        <v>5</v>
-      </c>
-      <c r="C11" s="12">
+      <c r="B11" s="18">
+        <v>5</v>
+      </c>
+      <c r="C11" s="18">
         <v>5</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F11" s="6"/>
     </row>
@@ -1628,76 +1667,76 @@
       <c r="A12" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="12">
-        <v>5</v>
-      </c>
-      <c r="C12" s="12">
+      <c r="B12" s="18">
+        <v>5</v>
+      </c>
+      <c r="C12" s="18">
         <v>5</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
         <v>25</v>
       </c>
-      <c r="B13" s="12">
-        <v>5</v>
-      </c>
-      <c r="C13" s="12">
+      <c r="B13" s="18">
+        <v>5</v>
+      </c>
+      <c r="C13" s="18">
         <v>5</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
         <v>23</v>
       </c>
-      <c r="B14">
-        <v>10</v>
-      </c>
-      <c r="C14">
+      <c r="B14" s="17">
+        <v>10</v>
+      </c>
+      <c r="C14" s="17">
         <v>10</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="15" spans="1:6">
-      <c r="A15" s="15" t="s">
+      <c r="A15" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="B15" s="15">
+      <c r="B15" s="19">
         <f>10-10</f>
         <v>0</v>
       </c>
-      <c r="C15" s="15">
+      <c r="C15" s="19">
         <v>0</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B16" s="3">
+      <c r="B16" s="20">
         <f>SUM(B11:B15)</f>
         <v>25</v>
       </c>
-      <c r="C16" s="3">
+      <c r="C16" s="20">
         <f>SUM(C11:C15)</f>
         <v>25</v>
       </c>
       <c r="D16" s="13"/>
     </row>
     <row r="17" spans="1:6">
-      <c r="B17" s="3"/>
-      <c r="C17" s="3"/>
+      <c r="B17" s="20"/>
+      <c r="C17" s="20"/>
       <c r="D17" s="13"/>
       <c r="F17" s="6"/>
     </row>
@@ -1705,6 +1744,8 @@
       <c r="A18" s="8" t="s">
         <v>6</v>
       </c>
+      <c r="B18" s="17"/>
+      <c r="C18" s="17"/>
       <c r="D18" s="13"/>
       <c r="F18" s="6"/>
     </row>
@@ -1712,29 +1753,29 @@
       <c r="A19" t="s">
         <v>7</v>
       </c>
-      <c r="B19">
+      <c r="B19" s="17">
         <v>3</v>
       </c>
-      <c r="C19">
+      <c r="C19" s="17">
         <v>3</v>
       </c>
       <c r="D19" s="13" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F19" s="6"/>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" t="s">
+        <v>28</v>
+      </c>
+      <c r="B20" s="17">
+        <v>2</v>
+      </c>
+      <c r="C20" s="17">
+        <v>2</v>
+      </c>
+      <c r="D20" s="13" t="s">
         <v>29</v>
-      </c>
-      <c r="B20">
-        <v>2</v>
-      </c>
-      <c r="C20">
-        <v>2</v>
-      </c>
-      <c r="D20" s="13" t="s">
-        <v>30</v>
       </c>
       <c r="F20" s="6"/>
     </row>
@@ -1742,11 +1783,11 @@
       <c r="A21" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B21" s="3">
+      <c r="B21" s="20">
         <f>SUM(B19:B20)</f>
         <v>5</v>
       </c>
-      <c r="C21" s="3">
+      <c r="C21" s="20">
         <f>SUM(C19:C20)</f>
         <v>5</v>
       </c>
@@ -1755,6 +1796,8 @@
     </row>
     <row r="22" spans="1:6">
       <c r="A22" s="1"/>
+      <c r="B22" s="17"/>
+      <c r="C22" s="17"/>
       <c r="D22" s="13"/>
       <c r="F22" s="6"/>
     </row>
@@ -1762,11 +1805,11 @@
       <c r="A23" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="B23" s="10">
+      <c r="B23" s="21">
         <f>SUM(B7,B16,B21)</f>
         <v>40</v>
       </c>
-      <c r="C23" s="10">
+      <c r="C23" s="21">
         <f>SUM(C7,C16,C21)</f>
         <v>40</v>
       </c>
@@ -1789,10 +1832,12 @@
       <c r="F26" s="6"/>
     </row>
     <row r="27" spans="1:6">
-      <c r="A27" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D27" s="13"/>
+      <c r="A27" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="B27" s="16"/>
+      <c r="C27" s="16"/>
+      <c r="D27" s="16"/>
       <c r="F27" s="6"/>
     </row>
     <row r="28" spans="1:6">
@@ -1815,17 +1860,21 @@
     </row>
     <row r="30" spans="1:6">
       <c r="A30" t="s">
-        <v>5</v>
-      </c>
-      <c r="B30">
-        <v>10</v>
-      </c>
-      <c r="C30">
-        <v>10</v>
-      </c>
-      <c r="D30" s="13"/>
+        <v>32</v>
+      </c>
+      <c r="B30" s="17">
+        <v>10</v>
+      </c>
+      <c r="C30" s="17">
+        <v>10</v>
+      </c>
+      <c r="D30" s="13" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="31" spans="1:6">
+      <c r="B31" s="17"/>
+      <c r="C31" s="17"/>
       <c r="D31" s="13"/>
       <c r="F31" s="6"/>
     </row>
@@ -1833,6 +1882,8 @@
       <c r="A32" s="4" t="s">
         <v>21</v>
       </c>
+      <c r="B32" s="17"/>
+      <c r="C32" s="17"/>
       <c r="D32" s="13"/>
       <c r="F32" s="6"/>
     </row>
@@ -1840,127 +1891,141 @@
       <c r="A33" t="s">
         <v>8</v>
       </c>
+      <c r="B33" s="17"/>
+      <c r="C33" s="17"/>
       <c r="D33" s="13"/>
     </row>
     <row r="34" spans="1:6">
       <c r="A34" t="s">
         <v>22</v>
       </c>
-      <c r="B34">
-        <v>5</v>
-      </c>
-      <c r="C34">
-        <v>5</v>
-      </c>
-      <c r="D34" s="13"/>
+      <c r="B34" s="17">
+        <v>5</v>
+      </c>
+      <c r="C34" s="17">
+        <v>5</v>
+      </c>
+      <c r="D34" s="13" t="s">
+        <v>29</v>
+      </c>
       <c r="F34" s="6"/>
     </row>
     <row r="35" spans="1:6">
       <c r="A35" t="s">
         <v>14</v>
       </c>
-      <c r="B35">
-        <v>5</v>
-      </c>
-      <c r="C35">
-        <v>5</v>
-      </c>
-      <c r="D35" s="13"/>
+      <c r="B35" s="17">
+        <v>5</v>
+      </c>
+      <c r="C35" s="17">
+        <v>5</v>
+      </c>
+      <c r="D35" s="13" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="36" spans="1:6">
       <c r="A36" t="s">
         <v>26</v>
       </c>
-      <c r="B36" s="12">
-        <v>5</v>
-      </c>
-      <c r="C36" s="12">
-        <v>5</v>
-      </c>
-      <c r="D36" s="13"/>
+      <c r="B36" s="18">
+        <v>5</v>
+      </c>
+      <c r="C36" s="18">
+        <v>5</v>
+      </c>
+      <c r="D36" s="13" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="37" spans="1:6">
       <c r="A37" t="s">
         <v>23</v>
       </c>
-      <c r="B37">
-        <v>10</v>
-      </c>
-      <c r="C37">
-        <v>10</v>
-      </c>
-      <c r="D37" s="13"/>
+      <c r="B37" s="17">
+        <v>10</v>
+      </c>
+      <c r="C37" s="17">
+        <v>10</v>
+      </c>
+      <c r="D37" s="13" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="38" spans="1:6">
-      <c r="A38" t="s">
+      <c r="A38" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="B38">
-        <v>10</v>
-      </c>
-      <c r="C38">
-        <v>10</v>
-      </c>
-      <c r="D38" s="13"/>
+      <c r="B38" s="17"/>
+      <c r="C38" s="17"/>
+      <c r="D38" s="13" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="39" spans="1:6">
       <c r="A39" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B39" s="3">
+      <c r="B39" s="20">
         <f>SUM(B34:B38)</f>
-        <v>35</v>
-      </c>
-      <c r="C39" s="3">
+        <v>25</v>
+      </c>
+      <c r="C39" s="20">
         <f>SUM(C34:C38)</f>
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="D39" s="13"/>
     </row>
     <row r="40" spans="1:6">
-      <c r="B40" s="3"/>
-      <c r="C40" s="3"/>
+      <c r="B40" s="20"/>
+      <c r="C40" s="20"/>
       <c r="D40" s="13"/>
     </row>
     <row r="41" spans="1:6">
       <c r="A41" s="8" t="s">
         <v>6</v>
       </c>
+      <c r="B41" s="17"/>
+      <c r="C41" s="17"/>
       <c r="D41" s="13"/>
     </row>
     <row r="42" spans="1:6">
       <c r="A42" t="s">
         <v>7</v>
       </c>
-      <c r="B42">
+      <c r="B42" s="17">
         <v>3</v>
       </c>
-      <c r="C42">
+      <c r="C42" s="17">
         <v>3</v>
       </c>
-      <c r="D42" s="13"/>
+      <c r="D42" s="13" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="43" spans="1:6">
       <c r="A43" t="s">
+        <v>28</v>
+      </c>
+      <c r="B43" s="17">
+        <v>2</v>
+      </c>
+      <c r="C43" s="17">
+        <v>2</v>
+      </c>
+      <c r="D43" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="B43">
-        <v>2</v>
-      </c>
-      <c r="C43">
-        <v>2</v>
-      </c>
-      <c r="D43" s="13"/>
     </row>
     <row r="44" spans="1:6">
       <c r="A44" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B44" s="3">
+      <c r="B44" s="20">
         <f>SUM(B42:B43)</f>
         <v>5</v>
       </c>
-      <c r="C44" s="3">
+      <c r="C44" s="20">
         <f>SUM(C42:C43)</f>
         <v>5</v>
       </c>
@@ -1968,19 +2033,21 @@
     </row>
     <row r="45" spans="1:6">
       <c r="A45" s="1"/>
+      <c r="B45" s="17"/>
+      <c r="C45" s="17"/>
       <c r="D45" s="13"/>
     </row>
     <row r="46" spans="1:6">
       <c r="A46" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="B46" s="10">
+      <c r="B46" s="21">
         <f>SUM(B30,B39,B44)</f>
-        <v>50</v>
-      </c>
-      <c r="C46" s="10">
+        <v>40</v>
+      </c>
+      <c r="C46" s="21">
         <f>SUM(C30,C39,C44)</f>
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="D46" s="13"/>
     </row>
@@ -2001,10 +2068,12 @@
       <c r="D49" s="13"/>
     </row>
     <row r="50" spans="1:4">
-      <c r="A50" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="D50" s="13"/>
+      <c r="A50" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="B50" s="16"/>
+      <c r="C50" s="16"/>
+      <c r="D50" s="16"/>
     </row>
     <row r="51" spans="1:4">
       <c r="D51" s="13"/>
@@ -2025,151 +2094,173 @@
     </row>
     <row r="53" spans="1:4">
       <c r="A53" t="s">
-        <v>5</v>
-      </c>
-      <c r="B53">
-        <v>10</v>
-      </c>
-      <c r="C53">
-        <v>10</v>
-      </c>
-      <c r="D53" s="13"/>
+        <v>32</v>
+      </c>
+      <c r="B53" s="17">
+        <v>10</v>
+      </c>
+      <c r="C53" s="17">
+        <v>10</v>
+      </c>
+      <c r="D53" s="13" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="54" spans="1:4">
+      <c r="B54" s="17"/>
+      <c r="C54" s="17"/>
       <c r="D54" s="13"/>
     </row>
     <row r="55" spans="1:4" s="4" customFormat="1">
       <c r="A55" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B55"/>
-      <c r="C55"/>
-      <c r="D55" s="14"/>
+      <c r="B55" s="17"/>
+      <c r="C55" s="17"/>
+      <c r="D55" s="13"/>
     </row>
     <row r="56" spans="1:4">
       <c r="A56" t="s">
         <v>8</v>
       </c>
+      <c r="B56" s="17"/>
+      <c r="C56" s="17"/>
       <c r="D56" s="13"/>
     </row>
     <row r="57" spans="1:4">
       <c r="A57" t="s">
         <v>15</v>
       </c>
-      <c r="B57">
-        <v>5</v>
-      </c>
-      <c r="C57">
-        <v>5</v>
-      </c>
-      <c r="D57" s="13"/>
+      <c r="B57" s="17">
+        <v>5</v>
+      </c>
+      <c r="C57" s="17">
+        <v>5</v>
+      </c>
+      <c r="D57" s="13" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="58" spans="1:4">
       <c r="A58" t="s">
         <v>18</v>
       </c>
-      <c r="B58">
-        <v>5</v>
-      </c>
-      <c r="C58">
-        <v>5</v>
-      </c>
-      <c r="D58" s="13"/>
+      <c r="B58" s="17">
+        <v>5</v>
+      </c>
+      <c r="C58" s="17">
+        <v>5</v>
+      </c>
+      <c r="D58" s="13" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="59" spans="1:4">
       <c r="A59" t="s">
         <v>27</v>
       </c>
-      <c r="B59">
-        <v>5</v>
-      </c>
-      <c r="C59">
-        <v>5</v>
-      </c>
-      <c r="D59" s="13"/>
+      <c r="B59" s="17">
+        <v>5</v>
+      </c>
+      <c r="C59" s="17">
+        <v>5</v>
+      </c>
+      <c r="D59" s="13" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="60" spans="1:4">
       <c r="A60" t="s">
         <v>23</v>
       </c>
-      <c r="B60">
-        <v>10</v>
-      </c>
-      <c r="C60">
-        <v>10</v>
-      </c>
-      <c r="D60" s="13"/>
+      <c r="B60" s="17">
+        <v>10</v>
+      </c>
+      <c r="C60" s="17">
+        <v>10</v>
+      </c>
+      <c r="D60" s="13" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="61" spans="1:4">
-      <c r="A61" t="s">
+      <c r="A61" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="B61">
-        <v>10</v>
-      </c>
-      <c r="C61">
-        <v>10</v>
-      </c>
-      <c r="D61" s="13"/>
+      <c r="B61" s="19">
+        <v>0</v>
+      </c>
+      <c r="C61" s="19">
+        <v>0</v>
+      </c>
+      <c r="D61" s="13" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="62" spans="1:4">
       <c r="A62" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B62" s="3">
+      <c r="B62" s="20">
         <f>SUM(B57:B61)</f>
-        <v>35</v>
-      </c>
-      <c r="C62" s="3">
+        <v>25</v>
+      </c>
+      <c r="C62" s="20">
         <f>SUM(C57:C61)</f>
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="D62" s="13"/>
     </row>
     <row r="63" spans="1:4">
-      <c r="B63" s="3"/>
-      <c r="C63" s="3"/>
+      <c r="B63" s="20"/>
+      <c r="C63" s="20"/>
       <c r="D63" s="13"/>
     </row>
     <row r="64" spans="1:4">
       <c r="A64" s="8" t="s">
         <v>6</v>
       </c>
+      <c r="B64" s="17"/>
+      <c r="C64" s="17"/>
       <c r="D64" s="13"/>
     </row>
     <row r="65" spans="1:4">
       <c r="A65" t="s">
         <v>7</v>
       </c>
-      <c r="B65">
+      <c r="B65" s="17">
         <v>3</v>
       </c>
-      <c r="C65">
+      <c r="C65" s="17">
         <v>3</v>
       </c>
-      <c r="D65" s="13"/>
+      <c r="D65" s="13" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="66" spans="1:4">
       <c r="A66" t="s">
+        <v>28</v>
+      </c>
+      <c r="B66" s="17">
+        <v>2</v>
+      </c>
+      <c r="C66" s="17">
+        <v>2</v>
+      </c>
+      <c r="D66" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="B66">
-        <v>2</v>
-      </c>
-      <c r="C66">
-        <v>2</v>
-      </c>
-      <c r="D66" s="13"/>
     </row>
     <row r="67" spans="1:4">
       <c r="A67" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B67" s="3">
+      <c r="B67" s="20">
         <f>SUM(B65:B66)</f>
         <v>5</v>
       </c>
-      <c r="C67" s="3">
+      <c r="C67" s="20">
         <f>SUM(C65:C66)</f>
         <v>5</v>
       </c>
@@ -2177,24 +2268,31 @@
     </row>
     <row r="68" spans="1:4">
       <c r="A68" s="1"/>
+      <c r="B68" s="17"/>
+      <c r="C68" s="17"/>
       <c r="D68" s="13"/>
     </row>
     <row r="69" spans="1:4">
       <c r="A69" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="B69" s="10">
+      <c r="B69" s="21">
         <f>SUM(B53,B62,B67)</f>
-        <v>50</v>
-      </c>
-      <c r="C69" s="10">
+        <v>40</v>
+      </c>
+      <c r="C69" s="21">
         <f>SUM(C53,C62,C67)</f>
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="D69" s="13"/>
     </row>
   </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A27:D27"/>
+    <mergeCell ref="A50:D50"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>